<commit_message>
updated the theme and edit buttons
</commit_message>
<xml_diff>
--- a/Bid_Config_Files_Local/Bidportal_Userinfo_Local.xlsx
+++ b/Bid_Config_Files_Local/Bidportal_Userinfo_Local.xlsx
@@ -503,7 +503,7 @@
         <v>Yes</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-06-05T10:40:07.976Z</v>
+        <v>2026-06-08T11:14:51.439Z</v>
       </c>
     </row>
     <row r="4">
@@ -538,7 +538,7 @@
         <v>Yes</v>
       </c>
       <c r="K4" t="str">
-        <v>2026-06-05T11:16:17.141Z</v>
+        <v>2026-06-08T09:59:32.935Z</v>
       </c>
     </row>
     <row r="5">
@@ -573,7 +573,7 @@
         <v>Yes</v>
       </c>
       <c r="K5" t="str">
-        <v>2026-06-05T11:19:32.589Z</v>
+        <v>2026-06-08T11:14:29.538Z</v>
       </c>
     </row>
     <row r="6">
@@ -608,7 +608,7 @@
         <v>Yes</v>
       </c>
       <c r="K6" t="str">
-        <v>2026-06-05T05:50:46.463Z</v>
+        <v>2026-06-08T06:36:23.804Z</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
updated the login page UI
</commit_message>
<xml_diff>
--- a/Bid_Config_Files_Local/Bidportal_Userinfo_Local.xlsx
+++ b/Bid_Config_Files_Local/Bidportal_Userinfo_Local.xlsx
@@ -468,7 +468,7 @@
         <v>Yes</v>
       </c>
       <c r="K2" t="str">
-        <v>2026-06-02T09:39:38.158Z</v>
+        <v>2026-06-11T10:10:04.909Z</v>
       </c>
     </row>
     <row r="3">
@@ -503,7 +503,7 @@
         <v>Yes</v>
       </c>
       <c r="K3" t="str">
-        <v>2026-06-10T06:58:25.934Z</v>
+        <v>2026-06-11T03:40:55.264Z</v>
       </c>
     </row>
     <row r="4">
@@ -643,7 +643,7 @@
         <v>Yes</v>
       </c>
       <c r="K7" t="str">
-        <v>2026-06-05T10:24:52.613Z</v>
+        <v>2026-06-11T10:10:30.796Z</v>
       </c>
     </row>
     <row r="8">

</xml_diff>